<commit_message>
Masters vaults: the CoP table's names; drop WAG Straight hecht
The Masters vault rows now follow skills/ucg-masters-vaults.json (CoP):
its printed names ("Forward head spring", "Front handspring sw. with ¼
twist", the en dash in "Squat onto table – straight jump down"), its row
order and groups. WAG Straight hecht over table is gone: the CoP table
dropped it on 2026-10-06 (UCGM-wag-straight-hecht-over-table is retired).

IDs are pinned in build_data.py (MASTERS_IDS) instead of being slugged
from the name, so renames can't change them, and the build now fails on
any row that is neither a WG vault nor a pinned UCG Masters vault.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/source/Masters Vault Values.xlsx
+++ b/tools/source/Masters Vault Values.xlsx
@@ -666,14 +666,14 @@
     <row r="5" ht="15.75" customHeight="1" s="33">
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Squat onto table - straight jump down</t>
+          <t>Squat onto table – straight jump down</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="15">
-        <f>$C5+D$4</f>
+        <f>$C5+$D$4</f>
         <v/>
       </c>
       <c r="E5" s="16">
@@ -730,15 +730,15 @@
       <c r="I6" s="39" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="33">
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Straddle hecht over table</t>
         </is>
       </c>
-      <c r="C7" s="31" t="n">
+      <c r="C7" s="14" t="n">
         <v>0.5</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <f>$C7+$D$4</f>
         <v/>
       </c>
@@ -746,7 +746,7 @@
         <f>$C7+$E$4</f>
         <v/>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="16">
         <f>$C7+$F$4</f>
         <v/>
       </c>
@@ -754,7 +754,7 @@
         <f>$C7+$G$4</f>
         <v/>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="16">
         <f>$C7+$H$4</f>
         <v/>
       </c>
@@ -766,7 +766,7 @@
           <t>Tuck hecht over table</t>
         </is>
       </c>
-      <c r="C8" s="31" t="n">
+      <c r="C8" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="D8" s="16">
@@ -793,15 +793,15 @@
       <c r="J8" s="21" t="n"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="33">
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Pike hecht over table</t>
         </is>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="14" t="n">
         <v>1.1</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <f>$C9+$D$4</f>
         <v/>
       </c>
@@ -809,7 +809,7 @@
         <f>$C9+$E$4</f>
         <v/>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="16">
         <f>$C9+$F$4</f>
         <v/>
       </c>
@@ -817,7 +817,7 @@
         <f>$C9+$G$4</f>
         <v/>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="16">
         <f>$C9+$H$4</f>
         <v/>
       </c>
@@ -830,7 +830,7 @@
           <t>Straight hecht over table</t>
         </is>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="14" t="n">
         <v>1.6</v>
       </c>
       <c r="D10" s="16">
@@ -867,15 +867,15 @@
       <c r="I11" s="39" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="33">
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring  </t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="n">
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
         <v>1.2</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <f>$C12+$D$4</f>
         <v/>
       </c>
@@ -883,7 +883,7 @@
         <f>$C12+$E$4</f>
         <v/>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="16">
         <f>$C12+$F$4</f>
         <v/>
       </c>
@@ -891,19 +891,19 @@
         <f>$C12+$G$4</f>
         <v/>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="16">
         <f>$C12+$H$4</f>
         <v/>
       </c>
       <c r="I12" s="39" t="n"/>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="33">
-      <c r="B13" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring with 1/2 twist </t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="n">
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring with ½ twist</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
         <v>1.4</v>
       </c>
       <c r="D13" s="16">
@@ -929,15 +929,15 @@
       <c r="I13" s="39" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="33">
-      <c r="B14" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring with 1/1 twist </t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="n">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring with 1/1 twist</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
         <v>1.6</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <f>$C14+$D$4</f>
         <v/>
       </c>
@@ -945,7 +945,7 @@
         <f>$C14+$E$4</f>
         <v/>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="16">
         <f>$C14+$F$4</f>
         <v/>
       </c>
@@ -953,19 +953,19 @@
         <f>$C14+$G$4</f>
         <v/>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="16">
         <f>$C14+$H$4</f>
         <v/>
       </c>
       <c r="I14" s="39" t="n"/>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="33">
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring with 3/2 twist </t>
-        </is>
-      </c>
-      <c r="C15" s="31" t="n">
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring with 3/2 twist</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
         <v>1.8</v>
       </c>
       <c r="D15" s="16">
@@ -991,15 +991,15 @@
       <c r="I15" s="39" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="33">
-      <c r="B16" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. tucked </t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n">
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. tucked</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <f>$C16+$D$4</f>
         <v/>
       </c>
@@ -1007,7 +1007,7 @@
         <f>$C16+$E$4</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="16">
         <f>$C16+$F$4</f>
         <v/>
       </c>
@@ -1015,19 +1015,19 @@
         <f>$C16+$G$4</f>
         <v/>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="16">
         <f>$C16+$H$4</f>
         <v/>
       </c>
       <c r="I16" s="39" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="33">
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Front handspring and salto fwd. tucked with ½ twist</t>
         </is>
       </c>
-      <c r="C17" s="31" t="n">
+      <c r="C17" s="14" t="n">
         <v>2.4</v>
       </c>
       <c r="D17" s="16">
@@ -1053,15 +1053,15 @@
       <c r="I17" s="39" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="33">
-      <c r="B18" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. piked </t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="n">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. piked</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
         <v>2.4</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="16">
         <f>$C18+$D$4</f>
         <v/>
       </c>
@@ -1069,7 +1069,7 @@
         <f>$C18+$E$4</f>
         <v/>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="16">
         <f>$C18+$F$4</f>
         <v/>
       </c>
@@ -1077,19 +1077,19 @@
         <f>$C18+$G$4</f>
         <v/>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="16">
         <f>$C18+$H$4</f>
         <v/>
       </c>
       <c r="I18" s="39" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="33">
-      <c r="B19" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. piked with ½ twist </t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="n">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. piked with ½ twist</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n">
         <v>2.8</v>
       </c>
       <c r="D19" s="16">
@@ -1115,15 +1115,15 @@
       <c r="I19" s="39" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="33">
-      <c r="B20" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. stretched </t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="n">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. stretched</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n">
         <v>3.2</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="16">
         <f>$C20+$D$4</f>
         <v/>
       </c>
@@ -1131,7 +1131,7 @@
         <f>$C20+$E$4</f>
         <v/>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="16">
         <f>$C20+$F$4</f>
         <v/>
       </c>
@@ -1139,19 +1139,19 @@
         <f>$C20+$G$4</f>
         <v/>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="16">
         <f>$C20+$H$4</f>
         <v/>
       </c>
       <c r="I20" s="39" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="33">
-      <c r="B21" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. stretched wit ½ twist </t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="n">
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. stretched with ½ twist</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
         <v>3.6</v>
       </c>
       <c r="D21" s="16">
@@ -1187,15 +1187,15 @@
       <c r="I22" s="39" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="33">
-      <c r="B23" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring sw with 1/4 twist </t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="n">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring sw. with ¼ twist</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
         <v>1.2</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <f>$C23+$D$4</f>
         <v/>
       </c>
@@ -1203,7 +1203,7 @@
         <f>$C23+$E$4</f>
         <v/>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="16">
         <f>$C23+$F$4</f>
         <v/>
       </c>
@@ -1211,19 +1211,19 @@
         <f>$C23+$G$4</f>
         <v/>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="16">
         <f>$C23+$H$4</f>
         <v/>
       </c>
       <c r="I23" s="39" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="33">
-      <c r="B24" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring sw with 3/4 twist </t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="n">
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring sw. with ¾ twist</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
         <v>1.4</v>
       </c>
       <c r="D24" s="16">
@@ -1249,15 +1249,15 @@
       <c r="I24" s="39" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="33">
-      <c r="B25" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring sw with 5/4 twist </t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="n">
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring sw. with 5/4 twist</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="n">
         <v>1.6</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="16">
         <f>$C25+$D$4</f>
         <v/>
       </c>
@@ -1265,7 +1265,7 @@
         <f>$C25+$E$4</f>
         <v/>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="16">
         <f>$C25+$F$4</f>
         <v/>
       </c>
@@ -1273,19 +1273,19 @@
         <f>$C25+$G$4</f>
         <v/>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="16">
         <f>$C25+$H$4</f>
         <v/>
       </c>
       <c r="I25" s="39" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="33">
-      <c r="B26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara or Yurchenko tucked </t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="n">
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara or Yurchenko tucked</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="n">
         <v>1.8</v>
       </c>
       <c r="D26" s="16">
@@ -1311,15 +1311,15 @@
       <c r="I26" s="39" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="33">
-      <c r="B27" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara or Yurchenko piked </t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="n">
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara or Yurchenko piked</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="16">
         <f>$C27+$D$4</f>
         <v/>
       </c>
@@ -1327,7 +1327,7 @@
         <f>$C27+$E$4</f>
         <v/>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="16">
         <f>$C27+$F$4</f>
         <v/>
       </c>
@@ -1335,19 +1335,19 @@
         <f>$C27+$G$4</f>
         <v/>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="16">
         <f>$C27+$H$4</f>
         <v/>
       </c>
       <c r="I27" s="39" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="33">
-      <c r="B28" s="32" t="inlineStr">
-        <is>
-          <t>Tsukahara or Yurchenko tucked with 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="n">
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara or Yurchenko tucked with ½ twist</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
         <v>2</v>
       </c>
       <c r="D28" s="16">
@@ -1373,15 +1373,15 @@
       <c r="I28" s="39" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="33">
-      <c r="B29" s="28" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Tsukahara or Yurchenko tucked with 1/1 twist</t>
         </is>
       </c>
-      <c r="C29" s="31" t="n">
+      <c r="C29" s="14" t="n">
         <v>2.4</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="16">
         <f>$C29+$D$4</f>
         <v/>
       </c>
@@ -1389,7 +1389,7 @@
         <f>$C29+$E$4</f>
         <v/>
       </c>
-      <c r="F29" s="15">
+      <c r="F29" s="16">
         <f>$C29+$F$4</f>
         <v/>
       </c>
@@ -1397,19 +1397,19 @@
         <f>$C29+$G$4</f>
         <v/>
       </c>
-      <c r="H29" s="15">
+      <c r="H29" s="16">
         <f>$C29+$H$4</f>
         <v/>
       </c>
       <c r="I29" s="39" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="33">
-      <c r="B30" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara or Yurchenko stretched  </t>
-        </is>
-      </c>
-      <c r="C30" s="31" t="n">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara or Yurchenko stretched</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="n">
         <v>2.8</v>
       </c>
       <c r="D30" s="16">
@@ -1435,15 +1435,15 @@
       <c r="I30" s="39" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="33">
-      <c r="B31" s="28" t="inlineStr">
-        <is>
-          <t>Tsukahara or Yurchenko stretched with 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C31" s="31" t="n">
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara or Yurchenko stretched with ½ twist</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="n">
         <v>3.2</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="16">
         <f>$C31+$D$4</f>
         <v/>
       </c>
@@ -1451,7 +1451,7 @@
         <f>$C31+$E$4</f>
         <v/>
       </c>
-      <c r="F31" s="15">
+      <c r="F31" s="16">
         <f>$C31+$F$4</f>
         <v/>
       </c>
@@ -1459,19 +1459,19 @@
         <f>$C31+$G$4</f>
         <v/>
       </c>
-      <c r="H31" s="15">
+      <c r="H31" s="16">
         <f>$C31+$H$4</f>
         <v/>
       </c>
       <c r="I31" s="39" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="33">
-      <c r="B32" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara or Yurchenko stretched with 1/1 twist </t>
-        </is>
-      </c>
-      <c r="C32" s="31" t="n">
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara or Yurchenko stretched with 1/1 twist</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="n">
         <v>3.6</v>
       </c>
       <c r="D32" s="16">
@@ -2483,7 +2483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="B1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="33" min="1" max="1"/>
@@ -2571,30 +2571,30 @@
     <row r="5" ht="14.25" customHeight="1" s="33">
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Squat onto table - straight jump down</t>
+          <t>Squat onto table – straight jump down</t>
         </is>
       </c>
       <c r="C5" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="15">
-        <f>$C5+D$4</f>
+        <f>$C5+$D$4</f>
         <v/>
       </c>
       <c r="E5" s="16">
-        <f>$C5+E$4</f>
+        <f>$C5+$E$4</f>
         <v/>
       </c>
       <c r="F5" s="15">
-        <f>$C5+F$4</f>
+        <f>$C5+$F$4</f>
         <v/>
       </c>
       <c r="G5" s="16">
-        <f>$C5+G$4</f>
+        <f>$C5+$G$4</f>
         <v/>
       </c>
       <c r="H5" s="15">
-        <f>$C5+H$4</f>
+        <f>$C5+$H$4</f>
         <v/>
       </c>
       <c r="I5" s="38" t="inlineStr">
@@ -2613,29 +2613,29 @@
         <v>0</v>
       </c>
       <c r="D6" s="16">
-        <f>C6+$D$4</f>
+        <f>$C6+$D$4</f>
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>$C6+E$4</f>
+        <f>$C6+$E$4</f>
         <v/>
       </c>
       <c r="F6" s="16">
-        <f>$C6+F$4</f>
+        <f>$C6+$F$4</f>
         <v/>
       </c>
       <c r="G6" s="16">
-        <f>$C6+G$4</f>
+        <f>$C6+$G$4</f>
         <v/>
       </c>
       <c r="H6" s="16">
-        <f>$C6+H$4</f>
+        <f>$C6+$H$4</f>
         <v/>
       </c>
       <c r="I6" s="39" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1" s="33">
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Straddle hecht over table</t>
         </is>
@@ -2643,24 +2643,24 @@
       <c r="C7" s="31" t="n">
         <v>0.6</v>
       </c>
-      <c r="D7" s="15">
-        <f>C7+$D$4</f>
+      <c r="D7" s="16">
+        <f>$C7+$D$4</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>$C7+E$4</f>
-        <v/>
-      </c>
-      <c r="F7" s="15">
-        <f>$C7+F$4</f>
+        <f>$C7+$E$4</f>
+        <v/>
+      </c>
+      <c r="F7" s="16">
+        <f>$C7+$F$4</f>
         <v/>
       </c>
       <c r="G7" s="16">
-        <f>$C7+G$4</f>
-        <v/>
-      </c>
-      <c r="H7" s="15">
-        <f>$C7+H$4</f>
+        <f>$C7+$G$4</f>
+        <v/>
+      </c>
+      <c r="H7" s="16">
+        <f>$C7+$H$4</f>
         <v/>
       </c>
       <c r="I7" s="39" t="n"/>
@@ -2675,54 +2675,54 @@
         <v>0.6</v>
       </c>
       <c r="D8" s="16">
-        <f>C8+$D$4</f>
+        <f>$C8+$D$4</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>$C8+E$4</f>
+        <f>$C8+$E$4</f>
         <v/>
       </c>
       <c r="F8" s="16">
-        <f>$C8+F$4</f>
+        <f>$C8+$F$4</f>
         <v/>
       </c>
       <c r="G8" s="16">
-        <f>$C8+G$4</f>
+        <f>$C8+$G$4</f>
         <v/>
       </c>
       <c r="H8" s="16">
-        <f>$C8+H$4</f>
+        <f>$C8+$H$4</f>
         <v/>
       </c>
       <c r="I8" s="39" t="n"/>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="33">
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Pike hecht over table</t>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Forward head spring</t>
         </is>
       </c>
       <c r="C9" s="31" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="D9" s="15">
-        <f>C9+$D$4</f>
+        <v>0.8</v>
+      </c>
+      <c r="D9" s="16">
+        <f>$C9+$D$4</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>$C9+E$4</f>
-        <v/>
-      </c>
-      <c r="F9" s="15">
-        <f>$C9+F$4</f>
+        <f>$C9+$E$4</f>
+        <v/>
+      </c>
+      <c r="F9" s="16">
+        <f>$C9+$F$4</f>
         <v/>
       </c>
       <c r="G9" s="16">
-        <f>$C9+G$4</f>
-        <v/>
-      </c>
-      <c r="H9" s="15">
-        <f>$C9+H$4</f>
+        <f>$C9+$G$4</f>
+        <v/>
+      </c>
+      <c r="H9" s="16">
+        <f>$C9+$H$4</f>
         <v/>
       </c>
       <c r="I9" s="39" t="n"/>
@@ -2730,191 +2730,170 @@
     <row r="10" ht="14.25" customHeight="1" s="33">
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Straight hecht over table</t>
+          <t>Pike hecht over table</t>
         </is>
       </c>
       <c r="C10" s="31" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="D10" s="16">
-        <f>C10+$D$4</f>
+        <f>$C10+$D$4</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>$C10+E$4</f>
+        <f>$C10+$E$4</f>
         <v/>
       </c>
       <c r="F10" s="16">
-        <f>$C10+F$4</f>
+        <f>$C10+$F$4</f>
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>$C10+G$4</f>
+        <f>$C10+$G$4</f>
         <v/>
       </c>
       <c r="H10" s="16">
-        <f>$C10+H$4</f>
+        <f>$C10+$H$4</f>
         <v/>
       </c>
       <c r="I10" s="39" t="n"/>
     </row>
     <row r="11" ht="5.25" customHeight="1" s="33">
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Forward headspring</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D11" s="16">
-        <f>$C11+D$4</f>
-        <v/>
-      </c>
-      <c r="E11" s="16">
-        <f>$C11+E$4</f>
-        <v/>
-      </c>
-      <c r="F11" s="16">
-        <f>$C11+F$4</f>
-        <v/>
-      </c>
-      <c r="G11" s="16">
-        <f>$C11+G$4</f>
-        <v/>
-      </c>
-      <c r="H11" s="16">
-        <f>$C11+H$4</f>
-        <v/>
-      </c>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="15" t="n"/>
       <c r="I11" s="39" t="n"/>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="33">
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring  </t>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring</t>
         </is>
       </c>
       <c r="C12" s="31" t="n">
         <v>1.6</v>
       </c>
-      <c r="D12" s="15">
-        <f>C12+$D$4</f>
+      <c r="D12" s="16">
+        <f>$C12+$D$4</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>$C12+E$4</f>
-        <v/>
-      </c>
-      <c r="F12" s="15">
-        <f>$C12+F$4</f>
+        <f>$C12+$E$4</f>
+        <v/>
+      </c>
+      <c r="F12" s="16">
+        <f>$C12+$F$4</f>
         <v/>
       </c>
       <c r="G12" s="16">
-        <f>$C12+G$4</f>
-        <v/>
-      </c>
-      <c r="H12" s="15">
-        <f>$C12+H$4</f>
+        <f>$C12+$G$4</f>
+        <v/>
+      </c>
+      <c r="H12" s="16">
+        <f>$C12+$H$4</f>
         <v/>
       </c>
       <c r="I12" s="39" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="33">
-      <c r="B13" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring with 1/2 twist </t>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring with ½ twist</t>
         </is>
       </c>
       <c r="C13" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="16">
-        <f>C13+$D$4</f>
+        <f>$C13+$D$4</f>
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>$C13+E$4</f>
+        <f>$C13+$E$4</f>
         <v/>
       </c>
       <c r="F13" s="16">
-        <f>$C13+F$4</f>
+        <f>$C13+$F$4</f>
         <v/>
       </c>
       <c r="G13" s="16">
-        <f>$C13+G$4</f>
+        <f>$C13+$G$4</f>
         <v/>
       </c>
       <c r="H13" s="16">
-        <f>$C13+H$4</f>
+        <f>$C13+$H$4</f>
         <v/>
       </c>
       <c r="I13" s="39" t="n"/>
     </row>
     <row r="14" ht="14.25" customHeight="1" s="33">
-      <c r="B14" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring with 1/1 twist </t>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring with 1/1 twist</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
         <v>2.6</v>
       </c>
-      <c r="D14" s="15">
-        <f>C14+$D$4</f>
+      <c r="D14" s="16">
+        <f>$C14+$D$4</f>
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>$C14+E$4</f>
-        <v/>
-      </c>
-      <c r="F14" s="15">
-        <f>$C14+F$4</f>
+        <f>$C14+$E$4</f>
+        <v/>
+      </c>
+      <c r="F14" s="16">
+        <f>$C14+$F$4</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>$C14+G$4</f>
-        <v/>
-      </c>
-      <c r="H14" s="15">
-        <f>$C14+H$4</f>
+        <f>$C14+$G$4</f>
+        <v/>
+      </c>
+      <c r="H14" s="16">
+        <f>$C14+$H$4</f>
         <v/>
       </c>
       <c r="I14" s="39" t="n"/>
     </row>
     <row r="15" ht="14.25" customHeight="1" s="33">
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring with 3/2 twist </t>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring with 3/2 twist</t>
         </is>
       </c>
       <c r="C15" s="31" t="n">
         <v>3.2</v>
       </c>
       <c r="D15" s="16">
-        <f>C15+$D$4</f>
+        <f>$C15+$D$4</f>
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>$C15+E$4</f>
+        <f>$C15+$E$4</f>
         <v/>
       </c>
       <c r="F15" s="16">
-        <f>$C15+F$4</f>
+        <f>$C15+$F$4</f>
         <v/>
       </c>
       <c r="G15" s="16">
-        <f>$C15+G$4</f>
+        <f>$C15+$G$4</f>
         <v/>
       </c>
       <c r="H15" s="16">
-        <f>$C15+H$4</f>
+        <f>$C15+$H$4</f>
         <v/>
       </c>
       <c r="I15" s="39" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1" s="33">
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>Front handspring with ½ twist 1st phase</t>
         </is>
@@ -2922,30 +2901,30 @@
       <c r="C16" s="31" t="n">
         <v>1.6</v>
       </c>
-      <c r="D16" s="15">
-        <f>C16+$D$4</f>
+      <c r="D16" s="16">
+        <f>$C16+$D$4</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>$C16+E$4</f>
-        <v/>
-      </c>
-      <c r="F16" s="15">
-        <f>$C16+F$4</f>
+        <f>$C16+$E$4</f>
+        <v/>
+      </c>
+      <c r="F16" s="16">
+        <f>$C16+$F$4</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>$C16+G$4</f>
-        <v/>
-      </c>
-      <c r="H16" s="15">
-        <f>$C16+H$4</f>
+        <f>$C16+$G$4</f>
+        <v/>
+      </c>
+      <c r="H16" s="16">
+        <f>$C16+$H$4</f>
         <v/>
       </c>
       <c r="I16" s="39" t="n"/>
     </row>
     <row r="17" ht="14.25" customHeight="1" s="33">
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Front handspring with ½ twist 1st phase and ½ twist 2nd</t>
         </is>
@@ -2954,785 +2933,821 @@
         <v>2.4</v>
       </c>
       <c r="D17" s="16">
-        <f>C17+$D$4</f>
+        <f>$C17+$D$4</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>$C17+E$4</f>
+        <f>$C17+$E$4</f>
         <v/>
       </c>
       <c r="F17" s="16">
-        <f>$C17+F$4</f>
+        <f>$C17+$F$4</f>
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>$C17+G$4</f>
+        <f>$C17+$G$4</f>
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>$C17+H$4</f>
+        <f>$C17+$H$4</f>
         <v/>
       </c>
       <c r="I17" s="39" t="n"/>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="33">
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="39" t="n"/>
+    </row>
+    <row r="19" ht="14.25" customHeight="1" s="33">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>Yamashita</t>
         </is>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="C19" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="15">
-        <f>C18+$D$4</f>
-        <v/>
-      </c>
-      <c r="E18" s="16">
-        <f>$C18+E$4</f>
-        <v/>
-      </c>
-      <c r="F18" s="15">
-        <f>$C18+F$4</f>
-        <v/>
-      </c>
-      <c r="G18" s="16">
-        <f>$C18+G$4</f>
-        <v/>
-      </c>
-      <c r="H18" s="15">
-        <f>$C18+H$4</f>
-        <v/>
-      </c>
-      <c r="I18" s="39" t="n"/>
-    </row>
-    <row r="19" ht="14.25" customHeight="1" s="33">
-      <c r="B19" s="32" t="inlineStr">
-        <is>
-          <t>Yamashita 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="n">
+      <c r="D19" s="16">
+        <f>$C19+$D$4</f>
+        <v/>
+      </c>
+      <c r="E19" s="16">
+        <f>$C19+$E$4</f>
+        <v/>
+      </c>
+      <c r="F19" s="16">
+        <f>$C19+$F$4</f>
+        <v/>
+      </c>
+      <c r="G19" s="16">
+        <f>$C19+$G$4</f>
+        <v/>
+      </c>
+      <c r="H19" s="16">
+        <f>$C19+$H$4</f>
+        <v/>
+      </c>
+      <c r="I19" s="39" t="n"/>
+    </row>
+    <row r="20" ht="14.25" customHeight="1" s="33">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Yamashita ½ twist</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n">
         <v>2.4</v>
       </c>
-      <c r="D19" s="16">
-        <f>C19+$D$4</f>
-        <v/>
-      </c>
-      <c r="E19" s="16">
-        <f>$C19+E$4</f>
-        <v/>
-      </c>
-      <c r="F19" s="16">
-        <f>$C19+F$4</f>
-        <v/>
-      </c>
-      <c r="G19" s="16">
-        <f>$C19+G$4</f>
-        <v/>
-      </c>
-      <c r="H19" s="16">
-        <f>$C19+H$4</f>
-        <v/>
-      </c>
-      <c r="I19" s="39" t="n"/>
-    </row>
-    <row r="20" ht="14.25" customHeight="1" s="33">
-      <c r="B20" s="28" t="inlineStr">
+      <c r="D20" s="16">
+        <f>$C20+$D$4</f>
+        <v/>
+      </c>
+      <c r="E20" s="16">
+        <f>$C20+$E$4</f>
+        <v/>
+      </c>
+      <c r="F20" s="16">
+        <f>$C20+$F$4</f>
+        <v/>
+      </c>
+      <c r="G20" s="16">
+        <f>$C20+$G$4</f>
+        <v/>
+      </c>
+      <c r="H20" s="16">
+        <f>$C20+$H$4</f>
+        <v/>
+      </c>
+      <c r="I20" s="39" t="n"/>
+    </row>
+    <row r="21" ht="14.25" customHeight="1" s="33">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Yamashita 1/1 twist</t>
         </is>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C21" s="31" t="n">
         <v>2.8</v>
       </c>
-      <c r="D20" s="15">
-        <f>C20+$D$4</f>
-        <v/>
-      </c>
-      <c r="E20" s="16">
-        <f>$C20+E$4</f>
-        <v/>
-      </c>
-      <c r="F20" s="15">
-        <f>$C20+F$4</f>
-        <v/>
-      </c>
-      <c r="G20" s="16">
-        <f>$C20+G$4</f>
-        <v/>
-      </c>
-      <c r="H20" s="15">
-        <f>$C20+H$4</f>
-        <v/>
-      </c>
-      <c r="I20" s="39" t="n"/>
-    </row>
-    <row r="21" ht="14.25" customHeight="1" s="33">
-      <c r="B21" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. tucked </t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="n">
+      <c r="D21" s="16">
+        <f>$C21+$D$4</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>$C21+$E$4</f>
+        <v/>
+      </c>
+      <c r="F21" s="16">
+        <f>$C21+$F$4</f>
+        <v/>
+      </c>
+      <c r="G21" s="16">
+        <f>$C21+$G$4</f>
+        <v/>
+      </c>
+      <c r="H21" s="16">
+        <f>$C21+$H$4</f>
+        <v/>
+      </c>
+      <c r="I21" s="39" t="n"/>
+    </row>
+    <row r="22" ht="14.25" customHeight="1" s="33">
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="31" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="39" t="n"/>
+    </row>
+    <row r="23" ht="14.25" customHeight="1" s="33">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. tucked</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="n">
         <v>3.6</v>
       </c>
-      <c r="D21" s="16">
-        <f>C21+$D$4</f>
-        <v/>
-      </c>
-      <c r="E21" s="16">
-        <f>$C21+E$4</f>
-        <v/>
-      </c>
-      <c r="F21" s="16">
-        <f>$C21+F$4</f>
-        <v/>
-      </c>
-      <c r="G21" s="16">
-        <f>$C21+G$4</f>
-        <v/>
-      </c>
-      <c r="H21" s="16">
-        <f>$C21+H$4</f>
-        <v/>
-      </c>
-      <c r="I21" s="39" t="n"/>
-    </row>
-    <row r="22" ht="14.25" customHeight="1" s="33">
-      <c r="B22" s="28" t="inlineStr">
+      <c r="D23" s="16">
+        <f>$C23+$D$4</f>
+        <v/>
+      </c>
+      <c r="E23" s="16">
+        <f>$C23+$E$4</f>
+        <v/>
+      </c>
+      <c r="F23" s="16">
+        <f>$C23+$F$4</f>
+        <v/>
+      </c>
+      <c r="G23" s="16">
+        <f>$C23+$G$4</f>
+        <v/>
+      </c>
+      <c r="H23" s="16">
+        <f>$C23+$H$4</f>
+        <v/>
+      </c>
+      <c r="I23" s="39" t="n"/>
+    </row>
+    <row r="24" ht="14.25" customHeight="1" s="33">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Front handspring and salto fwd. tucked with ½ twist</t>
         </is>
       </c>
-      <c r="C22" s="31" t="n">
+      <c r="C24" s="31" t="n">
         <v>3.8</v>
       </c>
-      <c r="D22" s="15">
-        <f>C22+$D$4</f>
-        <v/>
-      </c>
-      <c r="E22" s="16">
-        <f>$C22+E$4</f>
-        <v/>
-      </c>
-      <c r="F22" s="15">
-        <f>$C22+F$4</f>
-        <v/>
-      </c>
-      <c r="G22" s="16">
-        <f>$C22+G$4</f>
-        <v/>
-      </c>
-      <c r="H22" s="15">
-        <f>$C22+H$4</f>
-        <v/>
-      </c>
-      <c r="I22" s="39" t="n"/>
-    </row>
-    <row r="23" ht="14.25" customHeight="1" s="33">
-      <c r="B23" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. piked </t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="n">
+      <c r="D24" s="16">
+        <f>$C24+$D$4</f>
+        <v/>
+      </c>
+      <c r="E24" s="16">
+        <f>$C24+$E$4</f>
+        <v/>
+      </c>
+      <c r="F24" s="16">
+        <f>$C24+$F$4</f>
+        <v/>
+      </c>
+      <c r="G24" s="16">
+        <f>$C24+$G$4</f>
+        <v/>
+      </c>
+      <c r="H24" s="16">
+        <f>$C24+$H$4</f>
+        <v/>
+      </c>
+      <c r="I24" s="39" t="n"/>
+    </row>
+    <row r="25" ht="5.25" customHeight="1" s="33">
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. piked</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="n">
         <v>3.8</v>
       </c>
-      <c r="D23" s="16">
-        <f>C23+$D$4</f>
-        <v/>
-      </c>
-      <c r="E23" s="16">
-        <f>$C23+E$4</f>
-        <v/>
-      </c>
-      <c r="F23" s="16">
-        <f>$C23+F$4</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
-        <f>$C23+G$4</f>
-        <v/>
-      </c>
-      <c r="H23" s="16">
-        <f>$C23+H$4</f>
-        <v/>
-      </c>
-      <c r="I23" s="39" t="n"/>
-    </row>
-    <row r="24" ht="14.25" customHeight="1" s="33">
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring and salto fwd. piked with ½ twist </t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="n">
+      <c r="D25" s="16">
+        <f>$C25+$D$4</f>
+        <v/>
+      </c>
+      <c r="E25" s="16">
+        <f>$C25+$E$4</f>
+        <v/>
+      </c>
+      <c r="F25" s="16">
+        <f>$C25+$F$4</f>
+        <v/>
+      </c>
+      <c r="G25" s="16">
+        <f>$C25+$G$4</f>
+        <v/>
+      </c>
+      <c r="H25" s="16">
+        <f>$C25+$H$4</f>
+        <v/>
+      </c>
+      <c r="I25" s="39" t="n"/>
+    </row>
+    <row r="26" ht="14.25" customHeight="1" s="33">
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring and salto fwd. piked with ½ twist</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="D24" s="15">
-        <f>C24+$D$4</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>$C24+E$4</f>
-        <v/>
-      </c>
-      <c r="F24" s="15">
-        <f>$C24+F$4</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
-        <f>$C24+G$4</f>
-        <v/>
-      </c>
-      <c r="H24" s="15">
-        <f>$C24+H$4</f>
-        <v/>
-      </c>
-      <c r="I24" s="39" t="n"/>
-    </row>
-    <row r="25" ht="5.25" customHeight="1" s="33">
-      <c r="B25" s="23" t="n"/>
-      <c r="C25" s="31" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="15" t="n"/>
-      <c r="I25" s="39" t="n"/>
-    </row>
-    <row r="26" ht="14.25" customHeight="1" s="33">
-      <c r="B26" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring sw with 1/4 twist </t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="n">
+      <c r="D26" s="16">
+        <f>$C26+$D$4</f>
+        <v/>
+      </c>
+      <c r="E26" s="16">
+        <f>$C26+$E$4</f>
+        <v/>
+      </c>
+      <c r="F26" s="16">
+        <f>$C26+$F$4</f>
+        <v/>
+      </c>
+      <c r="G26" s="16">
+        <f>$C26+$G$4</f>
+        <v/>
+      </c>
+      <c r="H26" s="16">
+        <f>$C26+$H$4</f>
+        <v/>
+      </c>
+      <c r="I26" s="39" t="n"/>
+    </row>
+    <row r="27" ht="14.25" customHeight="1" s="33">
+      <c r="B27" s="23" t="n"/>
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="39" t="n"/>
+    </row>
+    <row r="28" ht="14.25" customHeight="1" s="33">
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring sw. with ¼ twist</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="n">
         <v>1.6</v>
       </c>
-      <c r="D26" s="15">
-        <f>C26+$D$4</f>
-        <v/>
-      </c>
-      <c r="E26" s="16">
-        <f>$C26+E$4</f>
-        <v/>
-      </c>
-      <c r="F26" s="15">
-        <f>$C26+F$4</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
-        <f>$C26+G$4</f>
-        <v/>
-      </c>
-      <c r="H26" s="15">
-        <f>$C26+H$4</f>
-        <v/>
-      </c>
-      <c r="I26" s="39" t="n"/>
-    </row>
-    <row r="27" ht="14.25" customHeight="1" s="33">
-      <c r="B27" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring sw with 3/4 twist </t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="n">
+      <c r="D28" s="16">
+        <f>$C28+$D$4</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>$C28+$E$4</f>
+        <v/>
+      </c>
+      <c r="F28" s="16">
+        <f>$C28+$F$4</f>
+        <v/>
+      </c>
+      <c r="G28" s="16">
+        <f>$C28+$G$4</f>
+        <v/>
+      </c>
+      <c r="H28" s="16">
+        <f>$C28+$H$4</f>
+        <v/>
+      </c>
+      <c r="I28" s="39" t="n"/>
+    </row>
+    <row r="29" ht="14.25" customHeight="1" s="33">
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring sw. with ¾ twist</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="16">
-        <f>C27+$D$4</f>
-        <v/>
-      </c>
-      <c r="E27" s="16">
-        <f>$C27+E$4</f>
-        <v/>
-      </c>
-      <c r="F27" s="16">
-        <f>$C27+F$4</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
-        <f>$C27+G$4</f>
-        <v/>
-      </c>
-      <c r="H27" s="16">
-        <f>$C27+H$4</f>
-        <v/>
-      </c>
-      <c r="I27" s="39" t="n"/>
-    </row>
-    <row r="28" ht="14.25" customHeight="1" s="33">
-      <c r="B28" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front handspring sw with 5/4 twist </t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="n">
+      <c r="D29" s="16">
+        <f>$C29+$D$4</f>
+        <v/>
+      </c>
+      <c r="E29" s="16">
+        <f>$C29+$E$4</f>
+        <v/>
+      </c>
+      <c r="F29" s="16">
+        <f>$C29+$F$4</f>
+        <v/>
+      </c>
+      <c r="G29" s="16">
+        <f>$C29+$G$4</f>
+        <v/>
+      </c>
+      <c r="H29" s="16">
+        <f>$C29+$H$4</f>
+        <v/>
+      </c>
+      <c r="I29" s="39" t="n"/>
+    </row>
+    <row r="30" ht="14.25" customHeight="1" s="33">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>Front handspring sw. with 5/4 twist</t>
+        </is>
+      </c>
+      <c r="C30" s="31" t="n">
         <v>2.6</v>
       </c>
-      <c r="D28" s="15">
-        <f>C28+$D$4</f>
-        <v/>
-      </c>
-      <c r="E28" s="16">
-        <f>$C28+E$4</f>
-        <v/>
-      </c>
-      <c r="F28" s="15">
-        <f>$C28+F$4</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>$C28+G$4</f>
-        <v/>
-      </c>
-      <c r="H28" s="15">
-        <f>$C28+H$4</f>
-        <v/>
-      </c>
-      <c r="I28" s="39" t="n"/>
-    </row>
-    <row r="29" ht="14.25" customHeight="1" s="33">
-      <c r="B29" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yurchenko tucked </t>
-        </is>
-      </c>
-      <c r="C29" s="31" t="n">
+      <c r="D30" s="16">
+        <f>$C30+$D$4</f>
+        <v/>
+      </c>
+      <c r="E30" s="16">
+        <f>$C30+$E$4</f>
+        <v/>
+      </c>
+      <c r="F30" s="16">
+        <f>$C30+$F$4</f>
+        <v/>
+      </c>
+      <c r="G30" s="16">
+        <f>$C30+$G$4</f>
+        <v/>
+      </c>
+      <c r="H30" s="16">
+        <f>$C30+$H$4</f>
+        <v/>
+      </c>
+      <c r="I30" s="39" t="n"/>
+    </row>
+    <row r="31" ht="14.25" customHeight="1" s="33">
+      <c r="B31" s="23" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="15" t="n"/>
+      <c r="I31" s="39" t="n"/>
+    </row>
+    <row r="32" ht="14.25" customHeight="1" s="33">
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>Yurchenko tucked</t>
+        </is>
+      </c>
+      <c r="C32" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="D29" s="16">
-        <f>C29+$D$4</f>
-        <v/>
-      </c>
-      <c r="E29" s="16">
-        <f>$C29+E$4</f>
-        <v/>
-      </c>
-      <c r="F29" s="16">
-        <f>$C29+F$4</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
-        <f>$C29+G$4</f>
-        <v/>
-      </c>
-      <c r="H29" s="16">
-        <f>$C29+H$4</f>
-        <v/>
-      </c>
-      <c r="I29" s="39" t="n"/>
-    </row>
-    <row r="30" ht="14.25" customHeight="1" s="33">
-      <c r="B30" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yurchenko piked </t>
-        </is>
-      </c>
-      <c r="C30" s="31" t="n">
+      <c r="D32" s="16">
+        <f>$C32+$D$4</f>
+        <v/>
+      </c>
+      <c r="E32" s="16">
+        <f>$C32+$E$4</f>
+        <v/>
+      </c>
+      <c r="F32" s="16">
+        <f>$C32+$F$4</f>
+        <v/>
+      </c>
+      <c r="G32" s="16">
+        <f>$C32+$G$4</f>
+        <v/>
+      </c>
+      <c r="H32" s="16">
+        <f>$C32+$H$4</f>
+        <v/>
+      </c>
+      <c r="I32" s="39" t="n"/>
+    </row>
+    <row r="33" ht="14.25" customHeight="1" s="33">
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>Yurchenko piked</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="n">
         <v>3.2</v>
       </c>
-      <c r="D30" s="15">
-        <f>C30+$D$4</f>
-        <v/>
-      </c>
-      <c r="E30" s="16">
-        <f>$C30+E$4</f>
-        <v/>
-      </c>
-      <c r="F30" s="15">
-        <f>$C30+F$4</f>
-        <v/>
-      </c>
-      <c r="G30" s="16">
-        <f>$C30+G$4</f>
-        <v/>
-      </c>
-      <c r="H30" s="15">
-        <f>$C30+H$4</f>
-        <v/>
-      </c>
-      <c r="I30" s="39" t="n"/>
-    </row>
-    <row r="31" ht="14.25" customHeight="1" s="33">
-      <c r="B31" s="32" t="inlineStr">
-        <is>
-          <t>Yurchenko tucked with 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C31" s="31" t="n">
+      <c r="D33" s="16">
+        <f>$C33+$D$4</f>
+        <v/>
+      </c>
+      <c r="E33" s="16">
+        <f>$C33+$E$4</f>
+        <v/>
+      </c>
+      <c r="F33" s="16">
+        <f>$C33+$F$4</f>
+        <v/>
+      </c>
+      <c r="G33" s="16">
+        <f>$C33+$G$4</f>
+        <v/>
+      </c>
+      <c r="H33" s="16">
+        <f>$C33+$H$4</f>
+        <v/>
+      </c>
+      <c r="I33" s="39" t="n"/>
+    </row>
+    <row r="34" ht="14.25" customHeight="1" s="33">
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>Yurchenko tucked with ½ twist</t>
+        </is>
+      </c>
+      <c r="C34" s="31" t="n">
         <v>3.2</v>
       </c>
-      <c r="D31" s="16">
-        <f>C31+$D$4</f>
-        <v/>
-      </c>
-      <c r="E31" s="16">
-        <f>$C31+E$4</f>
-        <v/>
-      </c>
-      <c r="F31" s="16">
-        <f>$C31+F$4</f>
-        <v/>
-      </c>
-      <c r="G31" s="16">
-        <f>$C31+G$4</f>
-        <v/>
-      </c>
-      <c r="H31" s="16">
-        <f>$C31+H$4</f>
-        <v/>
-      </c>
-      <c r="I31" s="39" t="n"/>
-    </row>
-    <row r="32" ht="14.25" customHeight="1" s="33">
-      <c r="B32" s="28" t="inlineStr">
+      <c r="D34" s="16">
+        <f>$C34+$D$4</f>
+        <v/>
+      </c>
+      <c r="E34" s="16">
+        <f>$C34+$E$4</f>
+        <v/>
+      </c>
+      <c r="F34" s="16">
+        <f>$C34+$F$4</f>
+        <v/>
+      </c>
+      <c r="G34" s="16">
+        <f>$C34+$G$4</f>
+        <v/>
+      </c>
+      <c r="H34" s="16">
+        <f>$C34+$H$4</f>
+        <v/>
+      </c>
+      <c r="I34" s="39" t="n"/>
+    </row>
+    <row r="35" ht="14.25" customHeight="1" s="33">
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>Yurchenko tucked with 1/1 twist</t>
         </is>
       </c>
-      <c r="C32" s="31" t="n">
+      <c r="C35" s="31" t="n">
         <v>3.6</v>
       </c>
-      <c r="D32" s="15">
-        <f>C32+$D$4</f>
-        <v/>
-      </c>
-      <c r="E32" s="16">
-        <f>$C32+E$4</f>
-        <v/>
-      </c>
-      <c r="F32" s="15">
-        <f>$C32+F$4</f>
-        <v/>
-      </c>
-      <c r="G32" s="16">
-        <f>$C32+G$4</f>
-        <v/>
-      </c>
-      <c r="H32" s="15">
-        <f>$C32+H$4</f>
-        <v/>
-      </c>
-      <c r="I32" s="39" t="n"/>
-    </row>
-    <row r="33" ht="14.25" customHeight="1" s="33">
-      <c r="B33" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yurchenko stretched  </t>
-        </is>
-      </c>
-      <c r="C33" s="31" t="n">
+      <c r="D35" s="16">
+        <f>$C35+$D$4</f>
+        <v/>
+      </c>
+      <c r="E35" s="16">
+        <f>$C35+$E$4</f>
+        <v/>
+      </c>
+      <c r="F35" s="16">
+        <f>$C35+$F$4</f>
+        <v/>
+      </c>
+      <c r="G35" s="16">
+        <f>$C35+$G$4</f>
+        <v/>
+      </c>
+      <c r="H35" s="16">
+        <f>$C35+$H$4</f>
+        <v/>
+      </c>
+      <c r="I35" s="39" t="n"/>
+    </row>
+    <row r="36" ht="14.25" customHeight="1" s="33">
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>Yurchenko stretched</t>
+        </is>
+      </c>
+      <c r="C36" s="31" t="n">
         <v>3.6</v>
       </c>
-      <c r="D33" s="16">
-        <f>C33+$D$4</f>
-        <v/>
-      </c>
-      <c r="E33" s="16">
-        <f>$C33+E$4</f>
-        <v/>
-      </c>
-      <c r="F33" s="16">
-        <f>$C33+F$4</f>
-        <v/>
-      </c>
-      <c r="G33" s="16">
-        <f>$C33+G$4</f>
-        <v/>
-      </c>
-      <c r="H33" s="16">
-        <f>$C33+H$4</f>
-        <v/>
-      </c>
-      <c r="I33" s="39" t="n"/>
-    </row>
-    <row r="34" ht="14.25" customHeight="1" s="33">
-      <c r="B34" s="28" t="inlineStr">
-        <is>
-          <t>Yurchenko stretched with 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C34" s="31" t="n">
+      <c r="D36" s="16">
+        <f>$C36+$D$4</f>
+        <v/>
+      </c>
+      <c r="E36" s="16">
+        <f>$C36+$E$4</f>
+        <v/>
+      </c>
+      <c r="F36" s="16">
+        <f>$C36+$F$4</f>
+        <v/>
+      </c>
+      <c r="G36" s="16">
+        <f>$C36+$G$4</f>
+        <v/>
+      </c>
+      <c r="H36" s="16">
+        <f>$C36+$H$4</f>
+        <v/>
+      </c>
+      <c r="I36" s="39" t="n"/>
+    </row>
+    <row r="37" ht="14.25" customHeight="1" s="33">
+      <c r="B37" s="18" t="inlineStr">
+        <is>
+          <t>Yurchenko stretched with ½ twist</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="n">
         <v>3.8</v>
       </c>
-      <c r="D34" s="15">
-        <f>C34+$D$4</f>
-        <v/>
-      </c>
-      <c r="E34" s="16">
-        <f>$C34+E$4</f>
-        <v/>
-      </c>
-      <c r="F34" s="15">
-        <f>$C34+F$4</f>
-        <v/>
-      </c>
-      <c r="G34" s="16">
-        <f>$C34+G$4</f>
-        <v/>
-      </c>
-      <c r="H34" s="15">
-        <f>$C34+H$4</f>
-        <v/>
-      </c>
-      <c r="I34" s="39" t="n"/>
-    </row>
-    <row r="35" ht="14.25" customHeight="1" s="33">
-      <c r="B35" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yurchenko stretched with 1/1 twist </t>
-        </is>
-      </c>
-      <c r="C35" s="31" t="n">
+      <c r="D37" s="16">
+        <f>$C37+$D$4</f>
+        <v/>
+      </c>
+      <c r="E37" s="16">
+        <f>$C37+$E$4</f>
+        <v/>
+      </c>
+      <c r="F37" s="16">
+        <f>$C37+$F$4</f>
+        <v/>
+      </c>
+      <c r="G37" s="16">
+        <f>$C37+$G$4</f>
+        <v/>
+      </c>
+      <c r="H37" s="16">
+        <f>$C37+$H$4</f>
+        <v/>
+      </c>
+      <c r="I37" s="39" t="n"/>
+    </row>
+    <row r="38" ht="14.25" customHeight="1" s="33">
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>Yurchenko stretched with 1/1 twist</t>
+        </is>
+      </c>
+      <c r="C38" s="31" t="n">
         <v>4.2</v>
       </c>
-      <c r="D35" s="16">
-        <f>C35+$D$4</f>
-        <v/>
-      </c>
-      <c r="E35" s="16">
-        <f>$C35+E$4</f>
-        <v/>
-      </c>
-      <c r="F35" s="16">
-        <f>$C35+F$4</f>
-        <v/>
-      </c>
-      <c r="G35" s="16">
-        <f>$C35+G$4</f>
-        <v/>
-      </c>
-      <c r="H35" s="16">
-        <f>$C35+H$4</f>
-        <v/>
-      </c>
-      <c r="I35" s="39" t="n"/>
-    </row>
-    <row r="36" ht="14.25" customHeight="1" s="33">
-      <c r="B36" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara tucked </t>
-        </is>
-      </c>
-      <c r="C36" s="31" t="n">
+      <c r="D38" s="16">
+        <f>$C38+$D$4</f>
+        <v/>
+      </c>
+      <c r="E38" s="16">
+        <f>$C38+$E$4</f>
+        <v/>
+      </c>
+      <c r="F38" s="16">
+        <f>$C38+$F$4</f>
+        <v/>
+      </c>
+      <c r="G38" s="16">
+        <f>$C38+$G$4</f>
+        <v/>
+      </c>
+      <c r="H38" s="16">
+        <f>$C38+$H$4</f>
+        <v/>
+      </c>
+      <c r="I38" s="39" t="n"/>
+    </row>
+    <row r="39" ht="14.25" customHeight="1" s="33">
+      <c r="B39" s="23" t="n"/>
+      <c r="C39" s="31" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="16" t="n"/>
+      <c r="H39" s="15" t="n"/>
+      <c r="I39" s="39" t="n"/>
+    </row>
+    <row r="40" ht="14.25" customHeight="1" s="33">
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara tucked</t>
+        </is>
+      </c>
+      <c r="C40" s="31" t="n">
         <v>3.2</v>
       </c>
-      <c r="D36" s="15">
-        <f>C36+$D$4</f>
-        <v/>
-      </c>
-      <c r="E36" s="16">
-        <f>$C36+E$4</f>
-        <v/>
-      </c>
-      <c r="F36" s="15">
-        <f>$C36+F$4</f>
-        <v/>
-      </c>
-      <c r="G36" s="16">
-        <f>$C36+G$4</f>
-        <v/>
-      </c>
-      <c r="H36" s="15">
-        <f>$C36+H$4</f>
-        <v/>
-      </c>
-      <c r="I36" s="39" t="n"/>
-    </row>
-    <row r="37" ht="14.25" customHeight="1" s="33">
-      <c r="B37" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara piked </t>
-        </is>
-      </c>
-      <c r="C37" s="31" t="n">
+      <c r="D40" s="16">
+        <f>$C40+$D$4</f>
+        <v/>
+      </c>
+      <c r="E40" s="16">
+        <f>$C40+$E$4</f>
+        <v/>
+      </c>
+      <c r="F40" s="16">
+        <f>$C40+$F$4</f>
+        <v/>
+      </c>
+      <c r="G40" s="16">
+        <f>$C40+$G$4</f>
+        <v/>
+      </c>
+      <c r="H40" s="16">
+        <f>$C40+$H$4</f>
+        <v/>
+      </c>
+      <c r="I40" s="39" t="n"/>
+    </row>
+    <row r="41" ht="14.25" customHeight="1" s="33">
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara piked</t>
+        </is>
+      </c>
+      <c r="C41" s="31" t="n">
         <v>3.4</v>
       </c>
-      <c r="D37" s="16">
-        <f>C37+$D$4</f>
-        <v/>
-      </c>
-      <c r="E37" s="16">
-        <f>$C37+E$4</f>
-        <v/>
-      </c>
-      <c r="F37" s="16">
-        <f>$C37+F$4</f>
-        <v/>
-      </c>
-      <c r="G37" s="16">
-        <f>$C37+G$4</f>
-        <v/>
-      </c>
-      <c r="H37" s="16">
-        <f>$C37+H$4</f>
-        <v/>
-      </c>
-      <c r="I37" s="39" t="n"/>
-    </row>
-    <row r="38" ht="14.25" customHeight="1" s="33">
-      <c r="B38" s="28" t="inlineStr">
-        <is>
-          <t>Tsukahara tucked with 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C38" s="31" t="n">
+      <c r="D41" s="16">
+        <f>$C41+$D$4</f>
+        <v/>
+      </c>
+      <c r="E41" s="16">
+        <f>$C41+$E$4</f>
+        <v/>
+      </c>
+      <c r="F41" s="16">
+        <f>$C41+$F$4</f>
+        <v/>
+      </c>
+      <c r="G41" s="16">
+        <f>$C41+$G$4</f>
+        <v/>
+      </c>
+      <c r="H41" s="16">
+        <f>$C41+$H$4</f>
+        <v/>
+      </c>
+      <c r="I41" s="39" t="n"/>
+    </row>
+    <row r="42" ht="14.25" customHeight="1" s="33">
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara tucked with ½ twist</t>
+        </is>
+      </c>
+      <c r="C42" s="31" t="n">
         <v>3.4</v>
       </c>
-      <c r="D38" s="15">
-        <f>C38+$D$4</f>
-        <v/>
-      </c>
-      <c r="E38" s="16">
-        <f>$C38+E$4</f>
-        <v/>
-      </c>
-      <c r="F38" s="15">
-        <f>$C38+F$4</f>
-        <v/>
-      </c>
-      <c r="G38" s="16">
-        <f>$C38+G$4</f>
-        <v/>
-      </c>
-      <c r="H38" s="15">
-        <f>$C38+H$4</f>
-        <v/>
-      </c>
-      <c r="I38" s="39" t="n"/>
-    </row>
-    <row r="39" ht="14.25" customHeight="1" s="33">
-      <c r="B39" s="32" t="inlineStr">
+      <c r="D42" s="16">
+        <f>$C42+$D$4</f>
+        <v/>
+      </c>
+      <c r="E42" s="16">
+        <f>$C42+$E$4</f>
+        <v/>
+      </c>
+      <c r="F42" s="16">
+        <f>$C42+$F$4</f>
+        <v/>
+      </c>
+      <c r="G42" s="16">
+        <f>$C42+$G$4</f>
+        <v/>
+      </c>
+      <c r="H42" s="16">
+        <f>$C42+$H$4</f>
+        <v/>
+      </c>
+      <c r="I42" s="39" t="n"/>
+    </row>
+    <row r="43" ht="14.25" customHeight="1" s="33">
+      <c r="B43" s="18" t="inlineStr">
         <is>
           <t>Tsukahara tucked with 1/1 twist</t>
         </is>
       </c>
-      <c r="C39" s="31" t="n">
+      <c r="C43" s="31" t="n">
         <v>3.8</v>
       </c>
-      <c r="D39" s="16">
-        <f>C39+$D$4</f>
-        <v/>
-      </c>
-      <c r="E39" s="16">
-        <f>$C39+E$4</f>
-        <v/>
-      </c>
-      <c r="F39" s="16">
-        <f>$C39+F$4</f>
-        <v/>
-      </c>
-      <c r="G39" s="16">
-        <f>$C39+G$4</f>
-        <v/>
-      </c>
-      <c r="H39" s="16">
-        <f>$C39+H$4</f>
-        <v/>
-      </c>
-      <c r="I39" s="39" t="n"/>
-    </row>
-    <row r="40" ht="14.25" customHeight="1" s="33">
-      <c r="B40" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara stretched  </t>
-        </is>
-      </c>
-      <c r="C40" s="31" t="n">
+      <c r="D43" s="16">
+        <f>$C43+$D$4</f>
+        <v/>
+      </c>
+      <c r="E43" s="16">
+        <f>$C43+$E$4</f>
+        <v/>
+      </c>
+      <c r="F43" s="16">
+        <f>$C43+$F$4</f>
+        <v/>
+      </c>
+      <c r="G43" s="16">
+        <f>$C43+$G$4</f>
+        <v/>
+      </c>
+      <c r="H43" s="16">
+        <f>$C43+$H$4</f>
+        <v/>
+      </c>
+      <c r="I43" s="39" t="n"/>
+    </row>
+    <row r="44" ht="14.25" customHeight="1" s="33">
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara stretched</t>
+        </is>
+      </c>
+      <c r="C44" s="31" t="n">
         <v>3.8</v>
       </c>
-      <c r="D40" s="15">
-        <f>C40+$D$4</f>
-        <v/>
-      </c>
-      <c r="E40" s="16">
-        <f>$C40+E$4</f>
-        <v/>
-      </c>
-      <c r="F40" s="15">
-        <f>$C40+F$4</f>
-        <v/>
-      </c>
-      <c r="G40" s="16">
-        <f>$C40+G$4</f>
-        <v/>
-      </c>
-      <c r="H40" s="15">
-        <f>$C40+H$4</f>
-        <v/>
-      </c>
-      <c r="I40" s="39" t="n"/>
-    </row>
-    <row r="41" ht="14.25" customHeight="1" s="33">
-      <c r="B41" s="32" t="inlineStr">
-        <is>
-          <t>Tsukahara stretched with 1/2 twist</t>
-        </is>
-      </c>
-      <c r="C41" s="31" t="n">
+      <c r="D44" s="16">
+        <f>$C44+$D$4</f>
+        <v/>
+      </c>
+      <c r="E44" s="16">
+        <f>$C44+$E$4</f>
+        <v/>
+      </c>
+      <c r="F44" s="16">
+        <f>$C44+$F$4</f>
+        <v/>
+      </c>
+      <c r="G44" s="16">
+        <f>$C44+$G$4</f>
+        <v/>
+      </c>
+      <c r="H44" s="16">
+        <f>$C44+$H$4</f>
+        <v/>
+      </c>
+      <c r="I44" s="39" t="n"/>
+    </row>
+    <row r="45" ht="14.25" customHeight="1" s="33">
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara stretched with ½ twist</t>
+        </is>
+      </c>
+      <c r="C45" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="D41" s="16">
-        <f>C41+$D$4</f>
-        <v/>
-      </c>
-      <c r="E41" s="16">
-        <f>$C41+E$4</f>
-        <v/>
-      </c>
-      <c r="F41" s="16">
-        <f>$C41+F$4</f>
-        <v/>
-      </c>
-      <c r="G41" s="16">
-        <f>$C41+G$4</f>
-        <v/>
-      </c>
-      <c r="H41" s="16">
-        <f>$C41+H$4</f>
-        <v/>
-      </c>
-      <c r="I41" s="39" t="n"/>
-    </row>
-    <row r="42" ht="14.25" customHeight="1" s="33">
-      <c r="B42" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsukahara stretched with 1/1 twist </t>
-        </is>
-      </c>
-      <c r="C42" s="31" t="n">
+      <c r="D45" s="16">
+        <f>$C45+$D$4</f>
+        <v/>
+      </c>
+      <c r="E45" s="16">
+        <f>$C45+$E$4</f>
+        <v/>
+      </c>
+      <c r="F45" s="16">
+        <f>$C45+$F$4</f>
+        <v/>
+      </c>
+      <c r="G45" s="16">
+        <f>$C45+$G$4</f>
+        <v/>
+      </c>
+      <c r="H45" s="16">
+        <f>$C45+$H$4</f>
+        <v/>
+      </c>
+      <c r="I45" s="39" t="n"/>
+    </row>
+    <row r="46" ht="14.25" customHeight="1" s="33">
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>Tsukahara stretched with 1/1 twist</t>
+        </is>
+      </c>
+      <c r="C46" s="31" t="n">
         <v>4.4</v>
       </c>
-      <c r="D42" s="15">
-        <f>C42+$D$4</f>
-        <v/>
-      </c>
-      <c r="E42" s="16">
-        <f>$C42+E$4</f>
-        <v/>
-      </c>
-      <c r="F42" s="15">
-        <f>$C42+F$4</f>
-        <v/>
-      </c>
-      <c r="G42" s="16">
-        <f>$C42+G$4</f>
-        <v/>
-      </c>
-      <c r="H42" s="15">
-        <f>$C42+H$4</f>
-        <v/>
-      </c>
-      <c r="I42" s="40" t="n"/>
-    </row>
-    <row r="43" ht="14.25" customHeight="1" s="33"/>
-    <row r="44" ht="14.25" customHeight="1" s="33"/>
-    <row r="45" ht="14.25" customHeight="1" s="33"/>
-    <row r="46" ht="14.25" customHeight="1" s="33"/>
+      <c r="D46" s="16">
+        <f>$C46+$D$4</f>
+        <v/>
+      </c>
+      <c r="E46" s="16">
+        <f>$C46+$E$4</f>
+        <v/>
+      </c>
+      <c r="F46" s="16">
+        <f>$C46+$F$4</f>
+        <v/>
+      </c>
+      <c r="G46" s="16">
+        <f>$C46+$G$4</f>
+        <v/>
+      </c>
+      <c r="H46" s="16">
+        <f>$C46+$H$4</f>
+        <v/>
+      </c>
+      <c r="I46" s="40" t="n"/>
+    </row>
     <row r="47" ht="14.25" customHeight="1" s="33"/>
     <row r="48" ht="14.25" customHeight="1" s="33"/>
     <row r="49" ht="14.25" customHeight="1" s="33"/>
@@ -4700,8 +4715,8 @@
     <row r="1011" ht="14.25" customHeight="1" s="33"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="I5:I46"/>
     <mergeCell ref="D2:H2"/>
-    <mergeCell ref="I5:I42"/>
     <mergeCell ref="B2:C3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>